<commit_message>
Improve Excel file handling by correctly adding member data and clearing dummy entries
Refactor Excel file writing logic to use `sheet_add_aoa` for data rows and ensure header rows are correctly initialized/maintained, while also resetting existing files to a clean state.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: fb83f075-83bf-4666-98f0-ea4bec10fd72
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 7f7355d1-5628-42f0-9a1d-beffd6b2d041
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/3a6f4480-5f60-41f1-9683-8e05aff8235c/fb83f075-83bf-4666-98f0-ea4bec10fd72/Aibtsmi
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,31 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
-    <col min="6" max="6" width="26.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="26.83203125" customWidth="1"/>
-    <col min="10" max="10" width="26.83203125" customWidth="1"/>
-    <col min="11" max="11" width="26.83203125" customWidth="1"/>
-    <col min="12" max="12" width="26.83203125" customWidth="1"/>
-    <col min="13" max="13" width="26.83203125" customWidth="1"/>
-    <col min="14" max="14" width="26.83203125" customWidth="1"/>
-    <col min="15" max="15" width="26.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>First name *</v>
+        <v>First name</v>
       </c>
       <c r="B1" t="str">
-        <v>Last name *</v>
+        <v>Last name</v>
       </c>
       <c r="C1" t="str">
         <v>Full name (Arabic)</v>
@@ -462,57 +445,13 @@
       <c r="O1" t="str">
         <v>ESC ID</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mohammad</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Al-Ahmad</v>
-      </c>
-      <c r="C2" t="str">
-        <v>محمد علي الأحمد</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Mohammad Al-Ahmad</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1985-06-15</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiology</v>
-      </c>
-      <c r="I2" t="str">
-        <v>example@email.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>0911234567</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Al-Mojtahed Hospital</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2020-01-01</v>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
+      <c r="P1" t="str">
+        <v>Submitted at</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve member form printing and prevent duplicate entries
Update print styles for a cleaner, professional look, disable email footers, and implement duplicate detection on member submissions.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 61aeea13-ec1a-4b13-8aab-23d387815147
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2aa21870-88bb-4262-b368-0720e6f97725
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2cea352b-fc04-48f7-b7b9-eaf259393ebb/61aeea13-ec1a-4b13-8aab-23d387815147/8ngODjy
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,109 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2025-09-05</v>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-05T18:29:23.690Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B3" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D3" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E3" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F3" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G3" t="str">
+        <v>male</v>
+      </c>
+      <c r="H3" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I3" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J3" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K3" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L3" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2025-09-05</v>
+      </c>
+      <c r="N3" t="str">
+        <v>original</v>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v>2026-05-05T18:31:00.770Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clear all data from membership form Excel files
Reset SCVA-Members-Template-EN.xlsx and نموذج-الأعضاء-عربي.xlsx to contain only header rows.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 61aeea13-ec1a-4b13-8aab-23d387815147
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 921df755-f172-4cd3-91c8-36ff65f77f45
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2cea352b-fc04-48f7-b7b9-eaf259393ebb/61aeea13-ec1a-4b13-8aab-23d387815147/8ngODjy
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,109 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2025-09-05</v>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-05T18:29:23.690Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B3" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D3" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E3" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F3" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G3" t="str">
-        <v>male</v>
-      </c>
-      <c r="H3" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I3" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J3" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K3" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L3" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M3" t="str">
-        <v>2025-09-05</v>
-      </c>
-      <c r="N3" t="str">
-        <v>original</v>
-      </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v>2026-05-05T18:31:00.770Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clear all data from English member template Excel file
Remove all data rows from the SCVA-Members-Template-EN.xlsx file, preserving only the header row.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 61aeea13-ec1a-4b13-8aab-23d387815147
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 470ab3d0-db45-420d-8f81-5e6d90e9c824
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2cea352b-fc04-48f7-b7b9-eaf259393ebb/61aeea13-ec1a-4b13-8aab-23d387815147/8ngODjy
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,59 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2025-09-05</v>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-05T18:59:38.076Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve email notifications by ensuring member data is correctly displayed
Update the workflow to use .first().json instead of .item.json in email templates for accurate data retrieval.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 61aeea13-ec1a-4b13-8aab-23d387815147
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9f802b61-3c04-4f85-996c-58e3aa748467
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2cea352b-fc04-48f7-b7b9-eaf259393ebb/61aeea13-ec1a-4b13-8aab-23d387815147/8ngODjy
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,59 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2025-09-05</v>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-05T18:59:38.076Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Excel template file for member data
Update the SCVA Members Excel template file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 61aeea13-ec1a-4b13-8aab-23d387815147
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 88545d96-b6b7-4271-acd2-7d256e096bc1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2cea352b-fc04-48f7-b7b9-eaf259393ebb/61aeea13-ec1a-4b13-8aab-23d387815147/8ngODjy
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,59 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2025-09-05</v>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-05T19:41:04.433Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update script to clear Excel data and use CommonJS modules
Rename `clear-excel.js` to `clear-excel.cjs` to support CommonJS modules with `require` syntax, and update instructions accordingly.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 61aeea13-ec1a-4b13-8aab-23d387815147
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6a881634-c7ef-4e6f-80d3-5d3be09cf7b2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2cea352b-fc04-48f7-b7b9-eaf259393ebb/61aeea13-ec1a-4b13-8aab-23d387815147/8ngODjy
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,59 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2025-09-05</v>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-05T19:41:04.433Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix empty email notifications and improve workflow reliability
Update workflow to correctly build and send email notifications by adjusting node positions, fixing data referencing, and optimizing HTTP request handling.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 61aeea13-ec1a-4b13-8aab-23d387815147
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2d12de7a-d097-45f3-bdbb-69e9a5f8b939
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2cea352b-fc04-48f7-b7b9-eaf259393ebb/61aeea13-ec1a-4b13-8aab-23d387815147/8ngODjy
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,59 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2025-09-05</v>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-05T19:57:27.633Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve AI node error handling and email content
Update the AI node in the workflow to gracefully handle missing API keys and ensure data is passed to email generation, preventing empty emails.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a54f8006-c148-4427-b135-ac0e7cb75f20
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9de8831f-d269-4ebd-b307-e81f880cca70
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/c4d58760-3d32-4049-bb81-9e806446f3f7/a54f8006-c148-4427-b135-ac0e7cb75f20/ua9tYb6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -475,19 +475,19 @@
         <v>cardiac_surgery</v>
       </c>
       <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
+        <v/>
       </c>
       <c r="J2" t="str">
         <v>+963933706403</v>
       </c>
       <c r="K2" t="str">
-        <v>damascus</v>
+        <v>admascus</v>
       </c>
       <c r="L2" t="str">
         <v>damascus</v>
       </c>
       <c r="M2" t="str">
-        <v>2025-09-05</v>
+        <v>2025-10-01</v>
       </c>
       <c r="N2" t="str">
         <v>original</v>
@@ -496,7 +496,7 @@
         <v/>
       </c>
       <c r="P2" t="str">
-        <v>2026-05-05T19:57:27.633Z</v>
+        <v>2026-05-05T20:50:41.568Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update AI node to use string concatenation for API calls
Refactor the AI node's JavaScript code within the n8n workflow JSON to use string concatenation instead of template literals for constructing API URLs and authorization headers, resolving syntax errors caused by shell interpretation of backticks.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a54f8006-c148-4427-b135-ac0e7cb75f20
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 10bf9395-b388-4ad7-acca-77c1a5fc0c1e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/c4d58760-3d32-4049-bb81-9e806446f3f7/a54f8006-c148-4427-b135-ac0e7cb75f20/3rz9vDc
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,59 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>admascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2025-10-01</v>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-05T21:07:26.271Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update email notifications to display correctly in Gmail
Update email generation to use inline styles for Gmail compatibility and fix a JavaScript syntax error in the AI node.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a54f8006-c148-4427-b135-ac0e7cb75f20
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: dac464fa-97cf-4acf-91f9-bb63579c51f4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/c4d58760-3d32-4049-bb81-9e806446f3f7/a54f8006-c148-4427-b135-ac0e7cb75f20/3rz9vDc
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,59 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>admascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-06T17:15:22.912Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update member template for form configuration
Update the SCVA Members Template Excel file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8535c23-4de2-4bd1-b14e-1cdf40c3c52c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: bb98b2d4-277e-4757-bfad-1116fdd398f5
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2bc78f45-813f-4a7a-bf2d-f7876258ac80/d8535c23-4de2-4bd1-b14e-1cdf40c3c52c/pBb41ir
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -475,19 +475,19 @@
         <v>cardiac_surgery</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>ibrahimsidawi@gmail.com</v>
       </c>
       <c r="J2" t="str">
         <v>+963933706403</v>
       </c>
       <c r="K2" t="str">
-        <v>admascus</v>
+        <v>damascus</v>
       </c>
       <c r="L2" t="str">
         <v>damascus</v>
       </c>
       <c r="M2" t="str">
-        <v>2025-10-01</v>
+        <v/>
       </c>
       <c r="N2" t="str">
         <v>original</v>
@@ -496,7 +496,7 @@
         <v/>
       </c>
       <c r="P2" t="str">
-        <v>2026-05-06T17:36:49.242Z</v>
+        <v>2026-05-06T18:19:26.603Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix error when building email content due to node naming Fixes a JavaScript syntax error in the 'Build Email HTML' node caused by incorrect newline escaping, ensuring emails are populated correctly.
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8535c23-4de2-4bd1-b14e-1cdf40c3c52c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8899c108-ea42-49f8-b15e-ae7fe397d03a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2bc78f45-813f-4a7a-bf2d-f7876258ac80/d8535c23-4de2-4bd1-b14e-1cdf40c3c52c/pBb41ir
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,59 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-06T18:38:10.578Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update member notification emails to ensure correct delivery and formatting
Fix email sending logic by referencing correct data sources and update workflow version.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8535c23-4de2-4bd1-b14e-1cdf40c3c52c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ce999db6-dcc5-4521-a4e7-d89a6207bb90
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2bc78f45-813f-4a7a-bf2d-f7876258ac80/d8535c23-4de2-4bd1-b14e-1cdf40c3c52c/pBb41ir
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,59 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-06T19:01:30.320Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update AI node to provide detailed logging and error handling
Rewrites the AI Analysis node to include comprehensive logging, remove the `canFetch` guard, and improve error handling for API responses.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8535c23-4de2-4bd1-b14e-1cdf40c3c52c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e738a66d-59a9-4dc4-8012-168295ef3e94
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2bc78f45-813f-4a7a-bf2d-f7876258ac80/d8535c23-4de2-4bd1-b14e-1cdf40c3c52c/AFspZtf
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,59 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-06T19:12:23.420Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update AI analysis to use compatible HTTP requests
Replace the `fetch` API with Node.js's built-in `https` module in the AI Analysis node for n8n compatibility.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8535c23-4de2-4bd1-b14e-1cdf40c3c52c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 64b0c4b2-0a06-4a76-b77e-e30f0c6e1015
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2bc78f45-813f-4a7a-bf2d-f7876258ac80/d8535c23-4de2-4bd1-b14e-1cdf40c3c52c/AFspZtf
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,59 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-06T19:43:21.158Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restructure AI processing to use dedicated nodes for prompt building and response handling
Replace the single AI analysis code node with a sequence of three nodes: a code node to build the AI prompt, an HTTP request node to call the AI service, and another code node to parse the AI response. Update server routes to inject the AI API key into the new prompt building node.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8535c23-4de2-4bd1-b14e-1cdf40c3c52c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4c85b60e-5be9-4cd8-80bd-085c8531cab6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2bc78f45-813f-4a7a-bf2d-f7876258ac80/d8535c23-4de2-4bd1-b14e-1cdf40c3c52c/AFspZtf
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,59 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-06T19:43:21.158Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add proposal document for Google Drive-based form system
Create a detailed proposal document outlining a system using Google Apps Script, Google Sheets, and Gmail to replicate the functionality of the current SCVA members template.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8535c23-4de2-4bd1-b14e-1cdf40c3c52c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 96fa5269-2299-4cf5-a264-d4913ab5faa5
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2bc78f45-813f-4a7a-bf2d-f7876258ac80/d8535c23-4de2-4bd1-b14e-1cdf40c3c52c/z8OhPuZ
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,59 @@
         <v>Submitted at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ibrahim</v>
+      </c>
+      <c r="B2" t="str">
+        <v>sidawi</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>mohammad ali</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>male</v>
+      </c>
+      <c r="H2" t="str">
+        <v>cardiac_surgery</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="L2" t="str">
+        <v>damascus</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>original</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-06T20:18:08.201Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Write new member data to both Arabic and English files
Refactor the `/api/public/append-excel` endpoint to always write to both the Arabic and English Excel files, regardless of the submission language, and perform duplicate detection across both files. Includes server-side translation maps for consistent labeling.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 05d607ca-8252-418b-a066-31438dd4eda5
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 3186404d-4805-4706-915d-1def6ab24b54
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e0e18a7a-58ce-429d-ba2b-70f8e0639f19/05d607ca-8252-418b-a066-31438dd4eda5/3T9GqjF
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
+++ b/docs/form_by_n8n/SCVA-Members-Template-EN.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,59 +449,9 @@
         <v>Submitted at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ibrahim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>sidawi</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ابراهيم الصيداوي</v>
-      </c>
-      <c r="D2" t="str">
-        <v>mohammad ali</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ibrahim sidawi</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1978-04-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>cardiac_surgery</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ibrahimsidawi@gmail.com</v>
-      </c>
-      <c r="J2" t="str">
-        <v>+963933706403</v>
-      </c>
-      <c r="K2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="L2" t="str">
-        <v>damascus</v>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v>original</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-05-06T20:18:08.201Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>